<commit_message>
feat: enhance experiment reliability with cloud sync and back navigation
</commit_message>
<xml_diff>
--- a/data/llm_cfs_report_questions_50.xlsx
+++ b/data/llm_cfs_report_questions_50.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/JackWu/git_project/crc-streamlit-app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB242672-9C63-9847-AF0E-6FB5B5342554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6594D502-70CF-0443-8BE5-0E305784D1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="620" windowWidth="38400" windowHeight="20980" xr2:uid="{6CBA2F91-21DC-2F40-AEAC-6FED94901F29}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16200" xr2:uid="{6CBA2F91-21DC-2F40-AEAC-6FED94901F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34588,7 +34589,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -34605,7 +34606,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -34654,16 +34655,19 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
@@ -35040,37 +35044,37 @@
         <v>192</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="22" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A4" s="18" t="s">
+    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="22" customFormat="1" ht="379" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
+    <row r="5" spans="1:5" ht="379" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="4" t="s">
         <v>193</v>
       </c>
     </row>
@@ -35142,54 +35146,54 @@
         <v>190</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="22" customFormat="1" ht="323" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+    <row r="10" spans="1:5" ht="323" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="22" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A11" s="18" t="s">
+    <row r="11" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="22" customFormat="1" ht="323" x14ac:dyDescent="0.2">
-      <c r="A12" s="18" t="s">
+    <row r="12" spans="1:5" ht="323" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="4" t="s">
         <v>191</v>
       </c>
     </row>
@@ -35295,20 +35299,20 @@
         <v>193</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="22" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A19" s="18" t="s">
+    <row r="19" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="D19" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="4" t="s">
         <v>191</v>
       </c>
     </row>
@@ -35380,20 +35384,20 @@
         <v>190</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="22" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A24" s="18" t="s">
+    <row r="24" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="D24" s="21" t="s">
+      <c r="D24" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="4" t="s">
         <v>191</v>
       </c>
     </row>
@@ -35465,37 +35469,37 @@
         <v>190</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="22" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A29" s="18" t="s">
+    <row r="29" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="E29" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="22" customFormat="1" ht="404" x14ac:dyDescent="0.2">
-      <c r="A30" s="18" t="s">
+    <row r="30" spans="1:5" ht="404" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C30" s="20" t="s">
+      <c r="C30" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="4" t="s">
         <v>191</v>
       </c>
     </row>
@@ -35584,37 +35588,37 @@
         <v>193</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="22" customFormat="1" ht="404" x14ac:dyDescent="0.2">
-      <c r="A36" s="18" t="s">
+    <row r="36" spans="1:5" ht="404" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B36" s="19" t="s">
+      <c r="B36" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="20" t="s">
+      <c r="C36" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D36" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="E36" s="20" t="s">
+      <c r="E36" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="22" customFormat="1" ht="352" x14ac:dyDescent="0.2">
-      <c r="A37" s="18" t="s">
+    <row r="37" spans="1:5" ht="349" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B37" s="19" t="s">
+      <c r="B37" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C37" s="20" t="s">
+      <c r="C37" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="D37" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E37" s="20" t="s">
+      <c r="E37" s="4" t="s">
         <v>191</v>
       </c>
     </row>
@@ -35635,20 +35639,20 @@
         <v>191</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="22" customFormat="1" ht="365" x14ac:dyDescent="0.2">
-      <c r="A39" s="18" t="s">
+    <row r="39" spans="1:5" ht="365" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B39" s="19" t="s">
+      <c r="B39" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C39" s="20" t="s">
+      <c r="C39" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="D39" s="21" t="s">
+      <c r="D39" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="E39" s="20" t="s">
+      <c r="E39" s="4" t="s">
         <v>191</v>
       </c>
     </row>
@@ -35669,20 +35673,20 @@
         <v>190</v>
       </c>
     </row>
-    <row r="41" spans="1:5" s="9" customFormat="1" ht="379" x14ac:dyDescent="0.2">
-      <c r="A41" s="5" t="s">
+    <row r="41" spans="1:5" s="23" customFormat="1" ht="379" x14ac:dyDescent="0.2">
+      <c r="A41" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="D41" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="E41" s="7" t="s">
+      <c r="E41" s="21" t="s">
         <v>192</v>
       </c>
     </row>
@@ -35703,37 +35707,37 @@
         <v>190</v>
       </c>
     </row>
-    <row r="43" spans="1:5" s="22" customFormat="1" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A43" s="18" t="s">
+    <row r="43" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="19" t="s">
+      <c r="B43" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C43" s="20" t="s">
+      <c r="C43" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="D43" s="21" t="s">
+      <c r="D43" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="E43" s="20" t="s">
+      <c r="E43" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="44" spans="1:5" s="22" customFormat="1" ht="365" x14ac:dyDescent="0.2">
-      <c r="A44" s="18" t="s">
+    <row r="44" spans="1:5" ht="365" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C44" s="20" t="s">
+      <c r="C44" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D44" s="21" t="s">
+      <c r="D44" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="E44" s="19" t="s">
+      <c r="E44" s="3" t="s">
         <v>194</v>
       </c>
     </row>
@@ -35805,20 +35809,20 @@
         <v>190</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="22" customFormat="1" ht="362" x14ac:dyDescent="0.2">
-      <c r="A49" s="18" t="s">
+    <row r="49" spans="1:5" ht="362" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B49" s="19" t="s">
+      <c r="B49" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C49" s="20" t="s">
+      <c r="C49" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="D49" s="21" t="s">
+      <c r="D49" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="E49" s="20" t="s">
+      <c r="E49" s="4" t="s">
         <v>191</v>
       </c>
     </row>

</xml_diff>